<commit_message>
Update C&P case. Other minor fixes.
</commit_message>
<xml_diff>
--- a/examples/HFP_chris+pat.xlsx
+++ b/examples/HFP_chris+pat.xlsx
@@ -508,85 +508,85 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="n">
+        <v>160000</v>
+      </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
+      <c r="F2" t="n">
+        <v>26000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="n">
+        <v>165000</v>
+      </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
+      <c r="F3" t="n">
+        <v>27000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="n">
+        <v>170000</v>
+      </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
+      <c r="F4" t="n">
+        <v>30000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>2024</v>
       </c>
+      <c r="B5" t="n">
+        <v>155000</v>
+      </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
+      <c r="F5" t="n">
+        <v>30500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>2025</v>
       </c>
+      <c r="B6" t="n">
+        <v>130000</v>
+      </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
+      <c r="F6" t="n">
+        <v>31000</v>
       </c>
     </row>
     <row r="7">
@@ -603,10 +603,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>23000</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
+        <v>29300</v>
       </c>
     </row>
     <row r="8">
@@ -614,7 +611,7 @@
         <v>2027</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -623,26 +620,17 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
+        <v>29300</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>2028</v>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -656,9 +644,6 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -670,9 +655,6 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -684,9 +666,6 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -698,9 +677,6 @@
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -712,9 +688,6 @@
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -726,9 +699,6 @@
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -740,9 +710,6 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -754,9 +721,6 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -768,9 +732,6 @@
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -782,9 +743,6 @@
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -796,9 +754,6 @@
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -810,9 +765,6 @@
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -824,9 +776,6 @@
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -838,9 +787,6 @@
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -852,9 +798,6 @@
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -866,9 +809,6 @@
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -880,9 +820,6 @@
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -894,9 +831,6 @@
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -908,9 +842,6 @@
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -922,9 +853,6 @@
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -936,9 +864,6 @@
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -950,9 +875,6 @@
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -964,9 +886,6 @@
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -978,9 +897,6 @@
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -992,9 +908,6 @@
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1006,9 +919,6 @@
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1018,9 +928,6 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1104,85 +1011,85 @@
       <c r="A2" t="n">
         <v>2021</v>
       </c>
+      <c r="B2" t="n">
+        <v>68000</v>
+      </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
+      <c r="F2" t="n">
+        <v>26000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2022</v>
       </c>
+      <c r="B3" t="n">
+        <v>72000</v>
+      </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
+      <c r="F3" t="n">
+        <v>27000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>2023</v>
       </c>
+      <c r="B4" t="n">
+        <v>75000</v>
+      </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
+      <c r="F4" t="n">
+        <v>30000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>2024</v>
       </c>
+      <c r="B5" t="n">
+        <v>78000</v>
+      </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>12000</v>
+      <c r="F5" t="n">
+        <v>30500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>2025</v>
       </c>
+      <c r="B6" t="n">
+        <v>80000</v>
+      </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
+      <c r="F6" t="n">
+        <v>31000</v>
       </c>
     </row>
     <row r="7">
@@ -1199,10 +1106,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>23000</v>
-      </c>
-      <c r="J7" t="n">
-        <v>4000</v>
+        <v>27700</v>
       </c>
     </row>
     <row r="8">
@@ -1219,10 +1123,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>23000</v>
-      </c>
-      <c r="J8" t="n">
-        <v>4000</v>
+        <v>27700</v>
       </c>
     </row>
     <row r="9">
@@ -1239,10 +1140,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>23000</v>
-      </c>
-      <c r="J9" t="n">
-        <v>4000</v>
+        <v>27900</v>
       </c>
     </row>
     <row r="10">
@@ -1255,9 +1153,6 @@
       <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="n">
-        <v>4000</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1269,9 +1164,6 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" t="n">
-        <v>4000</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1283,9 +1175,6 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1297,9 +1186,6 @@
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1311,9 +1197,6 @@
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1325,9 +1208,6 @@
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1339,9 +1219,6 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1353,9 +1230,6 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1367,9 +1241,6 @@
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1381,9 +1252,6 @@
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1395,9 +1263,6 @@
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1409,9 +1274,6 @@
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1423,9 +1285,6 @@
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1437,9 +1296,6 @@
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1451,9 +1307,6 @@
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1465,9 +1318,6 @@
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1479,9 +1329,6 @@
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1493,9 +1340,6 @@
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1507,9 +1351,6 @@
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1521,9 +1362,6 @@
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1535,9 +1373,6 @@
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1549,9 +1384,6 @@
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1563,9 +1395,6 @@
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1577,9 +1406,6 @@
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1591,9 +1417,6 @@
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1605,9 +1428,6 @@
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1619,9 +1439,6 @@
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1633,9 +1450,6 @@
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1647,9 +1461,6 @@
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="J38" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1659,9 +1470,6 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>